<commit_message>
README File for Product Sales Data Exploration & Output file Modified
</commit_message>
<xml_diff>
--- a/Sales_Data_Exploration/Excel_Product_Sales_Data_Exploration.xlsx
+++ b/Sales_Data_Exploration/Excel_Product_Sales_Data_Exploration.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Mani_Portfolio\Excel_Projects\Sales_Data_Exploration\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Mani_Portfolio\Excel-Projects\Sales_Data_Exploration\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E51710AF-25A8-4181-BFA8-353A1F581350}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{33B0E22C-70CF-4611-ABDB-E3EE358304DF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="777" xr2:uid="{D316CDA9-901C-489C-8901-42D27F55E62A}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="24240" windowHeight="13020" tabRatio="777" xr2:uid="{D316CDA9-901C-489C-8901-42D27F55E62A}"/>
   </bookViews>
   <sheets>
     <sheet name="Sales_DB_Dataset" sheetId="1" r:id="rId1"/>
@@ -546,11 +546,13 @@
       <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>

</xml_diff>